<commit_message>
Actualizacao do grafico sobre Desistencia apos Grants
</commit_message>
<xml_diff>
--- a/Lista_Grants_Mentoria.xlsx
+++ b/Lista_Grants_Mentoria.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://muvamozorg.sharepoint.com/sites/mis.drive/Documentos Partilhados/PROJECTOS/Sistema de Monitoria/NEXUS/2026/Dash_Nexus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1824" documentId="13_ncr:1_{54A37689-96D9-4BFE-9E28-8766A1F3212B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00C1E32F-FF37-4041-BE4A-74B33F06633F}"/>
+  <xr:revisionPtr revIDLastSave="1826" documentId="13_ncr:1_{54A37689-96D9-4BFE-9E28-8766A1F3212B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{72AE95A2-F412-4AFB-AC3C-7F3CDE75F6E9}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -1933,7 +1933,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{443F3E09-02E4-44F3-8428-F05D0B7CD6E5}" name="Table1" displayName="Table1" ref="A1:M450" totalsRowShown="0">
-  <autoFilter ref="A1:M450" xr:uid="{443F3E09-02E4-44F3-8428-F05D0B7CD6E5}"/>
+  <autoFilter ref="A1:M450" xr:uid="{443F3E09-02E4-44F3-8428-F05D0B7CD6E5}">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="Sim"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{DC8E42B1-C5DD-4FD8-BA52-9804B814B2E7}" name="Distrito"/>
     <tableColumn id="2" xr3:uid="{1E34E00E-4C4B-410D-9D66-0B462945AB80}" name="Facilitadores"/>
@@ -2233,24 +2239,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M450"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.44140625" customWidth="1"/>
-    <col min="3" max="3" width="49.5546875" customWidth="1"/>
-    <col min="4" max="4" width="18.5546875" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="17.88671875" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="36.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="50.5546875" customWidth="1"/>
-    <col min="13" max="13" width="66.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.42578125" customWidth="1"/>
+    <col min="3" max="3" width="49.5703125" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="17.85546875" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="50.5703125" customWidth="1"/>
+    <col min="13" max="13" width="66.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2291,7 +2297,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>97</v>
       </c>
@@ -2329,7 +2335,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>97</v>
       </c>
@@ -2367,7 +2373,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>97</v>
       </c>
@@ -2405,7 +2411,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>97</v>
       </c>
@@ -2443,7 +2449,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>97</v>
       </c>
@@ -2481,7 +2487,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>97</v>
       </c>
@@ -2519,7 +2525,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>97</v>
       </c>
@@ -2557,7 +2563,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>97</v>
       </c>
@@ -2595,7 +2601,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>97</v>
       </c>
@@ -2633,7 +2639,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>97</v>
       </c>
@@ -2671,7 +2677,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>97</v>
       </c>
@@ -2709,7 +2715,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>97</v>
       </c>
@@ -2747,7 +2753,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>97</v>
       </c>
@@ -2785,7 +2791,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>97</v>
       </c>
@@ -2823,7 +2829,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>97</v>
       </c>
@@ -2861,7 +2867,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>97</v>
       </c>
@@ -2899,7 +2905,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>97</v>
       </c>
@@ -2937,7 +2943,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>97</v>
       </c>
@@ -2975,7 +2981,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>97</v>
       </c>
@@ -3013,7 +3019,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>97</v>
       </c>
@@ -3051,7 +3057,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>97</v>
       </c>
@@ -3089,7 +3095,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>97</v>
       </c>
@@ -3127,7 +3133,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>97</v>
       </c>
@@ -3165,7 +3171,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>97</v>
       </c>
@@ -3203,7 +3209,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>97</v>
       </c>
@@ -3241,7 +3247,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>97</v>
       </c>
@@ -3279,7 +3285,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>97</v>
       </c>
@@ -3317,7 +3323,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>97</v>
       </c>
@@ -3355,7 +3361,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>97</v>
       </c>
@@ -3393,7 +3399,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>97</v>
       </c>
@@ -3431,7 +3437,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>97</v>
       </c>
@@ -3469,7 +3475,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>97</v>
       </c>
@@ -3507,7 +3513,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>97</v>
       </c>
@@ -3545,7 +3551,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>97</v>
       </c>
@@ -3583,7 +3589,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>97</v>
       </c>
@@ -3621,7 +3627,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>97</v>
       </c>
@@ -3659,7 +3665,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>97</v>
       </c>
@@ -3697,7 +3703,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>97</v>
       </c>
@@ -3735,7 +3741,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>97</v>
       </c>
@@ -3773,7 +3779,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>97</v>
       </c>
@@ -3811,7 +3817,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>97</v>
       </c>
@@ -3849,7 +3855,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>97</v>
       </c>
@@ -3887,7 +3893,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>97</v>
       </c>
@@ -3925,7 +3931,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>97</v>
       </c>
@@ -3963,7 +3969,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>97</v>
       </c>
@@ -4001,7 +4007,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>97</v>
       </c>
@@ -4039,7 +4045,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>97</v>
       </c>
@@ -4077,7 +4083,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>97</v>
       </c>
@@ -4115,7 +4121,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>97</v>
       </c>
@@ -4153,7 +4159,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>97</v>
       </c>
@@ -4191,7 +4197,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>97</v>
       </c>
@@ -4229,7 +4235,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>97</v>
       </c>
@@ -4267,7 +4273,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>97</v>
       </c>
@@ -4305,7 +4311,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>97</v>
       </c>
@@ -4343,7 +4349,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>97</v>
       </c>
@@ -4381,7 +4387,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>97</v>
       </c>
@@ -4419,7 +4425,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>97</v>
       </c>
@@ -4457,7 +4463,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>97</v>
       </c>
@@ -4495,7 +4501,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>97</v>
       </c>
@@ -4533,7 +4539,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>97</v>
       </c>
@@ -4571,7 +4577,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>97</v>
       </c>
@@ -4609,7 +4615,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>97</v>
       </c>
@@ -4647,7 +4653,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>97</v>
       </c>
@@ -4685,7 +4691,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>97</v>
       </c>
@@ -4723,7 +4729,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>97</v>
       </c>
@@ -4761,7 +4767,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>97</v>
       </c>
@@ -4799,7 +4805,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>97</v>
       </c>
@@ -4837,7 +4843,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>97</v>
       </c>
@@ -4875,7 +4881,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>97</v>
       </c>
@@ -4913,7 +4919,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>97</v>
       </c>
@@ -4951,7 +4957,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>97</v>
       </c>
@@ -4989,7 +4995,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>97</v>
       </c>
@@ -5027,7 +5033,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>97</v>
       </c>
@@ -5065,7 +5071,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>97</v>
       </c>
@@ -5103,7 +5109,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>97</v>
       </c>
@@ -5141,7 +5147,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>97</v>
       </c>
@@ -5179,7 +5185,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>97</v>
       </c>
@@ -5217,7 +5223,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>97</v>
       </c>
@@ -5255,7 +5261,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>97</v>
       </c>
@@ -5293,7 +5299,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>97</v>
       </c>
@@ -5331,7 +5337,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>97</v>
       </c>
@@ -5369,7 +5375,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>97</v>
       </c>
@@ -5407,7 +5413,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>97</v>
       </c>
@@ -5445,7 +5451,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>97</v>
       </c>
@@ -5483,7 +5489,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>97</v>
       </c>
@@ -5521,7 +5527,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>97</v>
       </c>
@@ -5559,7 +5565,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>97</v>
       </c>
@@ -5597,7 +5603,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>97</v>
       </c>
@@ -5635,7 +5641,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>97</v>
       </c>
@@ -5673,7 +5679,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>97</v>
       </c>
@@ -5711,7 +5717,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>97</v>
       </c>
@@ -5749,7 +5755,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>97</v>
       </c>
@@ -5787,7 +5793,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>97</v>
       </c>
@@ -5825,7 +5831,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>97</v>
       </c>
@@ -5863,7 +5869,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>97</v>
       </c>
@@ -5901,7 +5907,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>97</v>
       </c>
@@ -5939,7 +5945,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>97</v>
       </c>
@@ -5977,7 +5983,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>97</v>
       </c>
@@ -6015,7 +6021,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>97</v>
       </c>
@@ -6053,7 +6059,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>97</v>
       </c>
@@ -6091,7 +6097,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>97</v>
       </c>
@@ -6129,7 +6135,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>97</v>
       </c>
@@ -6167,7 +6173,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>97</v>
       </c>
@@ -6205,7 +6211,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>97</v>
       </c>
@@ -6243,7 +6249,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>97</v>
       </c>
@@ -6284,7 +6290,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>97</v>
       </c>
@@ -6322,7 +6328,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>97</v>
       </c>
@@ -6360,7 +6366,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>97</v>
       </c>
@@ -6398,7 +6404,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>97</v>
       </c>
@@ -6436,7 +6442,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>97</v>
       </c>
@@ -6474,7 +6480,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="112" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>97</v>
       </c>
@@ -6512,7 +6518,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>97</v>
       </c>
@@ -6550,7 +6556,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>97</v>
       </c>
@@ -6588,7 +6594,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>97</v>
       </c>
@@ -6626,7 +6632,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>97</v>
       </c>
@@ -6664,7 +6670,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>97</v>
       </c>
@@ -6702,7 +6708,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>97</v>
       </c>
@@ -6740,7 +6746,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>97</v>
       </c>
@@ -6778,7 +6784,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>97</v>
       </c>
@@ -6816,7 +6822,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>97</v>
       </c>
@@ -6854,7 +6860,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>97</v>
       </c>
@@ -6892,7 +6898,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>97</v>
       </c>
@@ -6930,7 +6936,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>97</v>
       </c>
@@ -6968,7 +6974,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>97</v>
       </c>
@@ -7006,7 +7012,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>97</v>
       </c>
@@ -7044,7 +7050,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>97</v>
       </c>
@@ -7082,7 +7088,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>97</v>
       </c>
@@ -7120,7 +7126,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>97</v>
       </c>
@@ -7158,7 +7164,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>97</v>
       </c>
@@ -7196,7 +7202,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>97</v>
       </c>
@@ -7234,7 +7240,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>97</v>
       </c>
@@ -7272,7 +7278,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>97</v>
       </c>
@@ -7310,7 +7316,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>97</v>
       </c>
@@ -7348,7 +7354,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>97</v>
       </c>
@@ -7386,7 +7392,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>97</v>
       </c>
@@ -7424,7 +7430,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>97</v>
       </c>
@@ -7462,7 +7468,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>97</v>
       </c>
@@ -7500,7 +7506,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>97</v>
       </c>
@@ -7538,7 +7544,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>97</v>
       </c>
@@ -7576,7 +7582,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>97</v>
       </c>
@@ -7614,7 +7620,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>97</v>
       </c>
@@ -7652,7 +7658,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>97</v>
       </c>
@@ -7690,7 +7696,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>97</v>
       </c>
@@ -7728,7 +7734,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>97</v>
       </c>
@@ -7766,7 +7772,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>97</v>
       </c>
@@ -7804,7 +7810,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>97</v>
       </c>
@@ -7842,7 +7848,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>97</v>
       </c>
@@ -7880,7 +7886,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>97</v>
       </c>
@@ -7918,7 +7924,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>97</v>
       </c>
@@ -7956,7 +7962,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>97</v>
       </c>
@@ -7994,7 +8000,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>97</v>
       </c>
@@ -8032,7 +8038,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>97</v>
       </c>
@@ -8070,7 +8076,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>97</v>
       </c>
@@ -8108,7 +8114,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>97</v>
       </c>
@@ -8146,7 +8152,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>97</v>
       </c>
@@ -8184,7 +8190,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>97</v>
       </c>
@@ -8222,7 +8228,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>97</v>
       </c>
@@ -8260,7 +8266,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>97</v>
       </c>
@@ -8298,7 +8304,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>97</v>
       </c>
@@ -8336,7 +8342,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>97</v>
       </c>
@@ -8374,7 +8380,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>97</v>
       </c>
@@ -8412,7 +8418,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>97</v>
       </c>
@@ -8450,7 +8456,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>97</v>
       </c>
@@ -8488,7 +8494,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>97</v>
       </c>
@@ -8526,7 +8532,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>97</v>
       </c>
@@ -8564,7 +8570,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>97</v>
       </c>
@@ -8602,7 +8608,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>97</v>
       </c>
@@ -8640,7 +8646,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>97</v>
       </c>
@@ -8678,7 +8684,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>97</v>
       </c>
@@ -8716,7 +8722,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>97</v>
       </c>
@@ -8754,7 +8760,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>97</v>
       </c>
@@ -8792,7 +8798,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>97</v>
       </c>
@@ -8830,7 +8836,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>97</v>
       </c>
@@ -8868,7 +8874,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>97</v>
       </c>
@@ -8906,7 +8912,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>97</v>
       </c>
@@ -8944,7 +8950,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>97</v>
       </c>
@@ -8982,7 +8988,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>97</v>
       </c>
@@ -9020,7 +9026,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>97</v>
       </c>
@@ -9058,7 +9064,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>97</v>
       </c>
@@ -9096,7 +9102,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>7</v>
       </c>
@@ -9134,7 +9140,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="182" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>7</v>
       </c>
@@ -9172,7 +9178,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="183" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>7</v>
       </c>
@@ -9210,7 +9216,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>7</v>
       </c>
@@ -9248,7 +9254,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="185" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>7</v>
       </c>
@@ -9286,7 +9292,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="186" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>7</v>
       </c>
@@ -9324,7 +9330,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="187" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>7</v>
       </c>
@@ -9362,7 +9368,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>7</v>
       </c>
@@ -9400,7 +9406,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>7</v>
       </c>
@@ -9438,7 +9444,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>7</v>
       </c>
@@ -9476,7 +9482,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>7</v>
       </c>
@@ -9514,7 +9520,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>7</v>
       </c>
@@ -9552,7 +9558,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="193" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>7</v>
       </c>
@@ -9590,7 +9596,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>7</v>
       </c>
@@ -9628,7 +9634,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="195" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>7</v>
       </c>
@@ -9666,7 +9672,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>7</v>
       </c>
@@ -9704,7 +9710,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="197" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>7</v>
       </c>
@@ -9742,7 +9748,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="198" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>7</v>
       </c>
@@ -9780,7 +9786,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="199" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>7</v>
       </c>
@@ -9818,7 +9824,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>7</v>
       </c>
@@ -9856,7 +9862,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="201" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>7</v>
       </c>
@@ -9894,7 +9900,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>7</v>
       </c>
@@ -9932,7 +9938,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="203" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>7</v>
       </c>
@@ -9970,7 +9976,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="204" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>7</v>
       </c>
@@ -10008,7 +10014,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="205" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>7</v>
       </c>
@@ -10046,7 +10052,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="206" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>7</v>
       </c>
@@ -10084,7 +10090,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="207" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>7</v>
       </c>
@@ -10122,7 +10128,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="208" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>7</v>
       </c>
@@ -10160,7 +10166,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="209" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>7</v>
       </c>
@@ -10198,7 +10204,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="210" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>7</v>
       </c>
@@ -10236,7 +10242,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="211" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>7</v>
       </c>
@@ -10274,7 +10280,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="212" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>7</v>
       </c>
@@ -10312,7 +10318,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="213" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>7</v>
       </c>
@@ -10350,7 +10356,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="214" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>7</v>
       </c>
@@ -10388,7 +10394,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="215" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>7</v>
       </c>
@@ -10426,7 +10432,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>7</v>
       </c>
@@ -10464,7 +10470,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="217" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>7</v>
       </c>
@@ -10502,7 +10508,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>7</v>
       </c>
@@ -10540,7 +10546,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="219" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>7</v>
       </c>
@@ -10578,7 +10584,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>7</v>
       </c>
@@ -10616,7 +10622,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="221" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>7</v>
       </c>
@@ -10654,7 +10660,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="222" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>7</v>
       </c>
@@ -10692,7 +10698,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="223" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>7</v>
       </c>
@@ -10730,7 +10736,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="224" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>7</v>
       </c>
@@ -10768,7 +10774,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="225" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>7</v>
       </c>
@@ -10806,7 +10812,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="226" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>7</v>
       </c>
@@ -10844,7 +10850,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="227" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>7</v>
       </c>
@@ -10882,7 +10888,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="228" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>7</v>
       </c>
@@ -10920,7 +10926,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="229" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>7</v>
       </c>
@@ -10958,7 +10964,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="230" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>7</v>
       </c>
@@ -10996,7 +11002,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="231" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>7</v>
       </c>
@@ -11034,7 +11040,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="232" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>7</v>
       </c>
@@ -11072,7 +11078,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="233" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>7</v>
       </c>
@@ -11110,7 +11116,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="234" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>7</v>
       </c>
@@ -11148,7 +11154,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="235" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>7</v>
       </c>
@@ -11186,7 +11192,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="236" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>7</v>
       </c>
@@ -11224,7 +11230,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="237" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>7</v>
       </c>
@@ -11262,7 +11268,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="238" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>7</v>
       </c>
@@ -11300,7 +11306,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="239" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>7</v>
       </c>
@@ -11338,7 +11344,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="240" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>7</v>
       </c>
@@ -11376,7 +11382,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="241" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>7</v>
       </c>
@@ -11414,7 +11420,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="242" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>7</v>
       </c>
@@ -11452,7 +11458,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="243" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>7</v>
       </c>
@@ -11490,7 +11496,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="244" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>7</v>
       </c>
@@ -11528,7 +11534,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="245" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>7</v>
       </c>
@@ -11566,7 +11572,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="246" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>7</v>
       </c>
@@ -11604,7 +11610,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="247" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>7</v>
       </c>
@@ -11642,7 +11648,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="248" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>7</v>
       </c>
@@ -11680,7 +11686,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="249" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>7</v>
       </c>
@@ -11718,7 +11724,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="250" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>7</v>
       </c>
@@ -11756,7 +11762,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="251" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>7</v>
       </c>
@@ -11794,7 +11800,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="252" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>7</v>
       </c>
@@ -11832,7 +11838,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="253" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>7</v>
       </c>
@@ -11870,7 +11876,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="254" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>7</v>
       </c>
@@ -11908,7 +11914,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="255" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>7</v>
       </c>
@@ -11946,7 +11952,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="256" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>7</v>
       </c>
@@ -11984,7 +11990,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="257" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>7</v>
       </c>
@@ -12022,7 +12028,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="258" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>7</v>
       </c>
@@ -12060,7 +12066,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="259" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>7</v>
       </c>
@@ -12098,7 +12104,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="260" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>7</v>
       </c>
@@ -12136,7 +12142,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="261" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>7</v>
       </c>
@@ -12174,7 +12180,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="262" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>7</v>
       </c>
@@ -12212,7 +12218,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="263" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>7</v>
       </c>
@@ -12250,7 +12256,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="264" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>7</v>
       </c>
@@ -12288,7 +12294,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="265" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>7</v>
       </c>
@@ -12326,7 +12332,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="266" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>7</v>
       </c>
@@ -12364,7 +12370,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="267" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>7</v>
       </c>
@@ -12402,7 +12408,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="268" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>7</v>
       </c>
@@ -12440,7 +12446,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="269" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>7</v>
       </c>
@@ -12478,7 +12484,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="270" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>7</v>
       </c>
@@ -12516,7 +12522,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="271" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>7</v>
       </c>
@@ -12554,7 +12560,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="272" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>7</v>
       </c>
@@ -12592,7 +12598,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="273" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>7</v>
       </c>
@@ -12630,7 +12636,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="274" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>7</v>
       </c>
@@ -12668,7 +12674,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="275" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>7</v>
       </c>
@@ -12706,7 +12712,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="276" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>7</v>
       </c>
@@ -12744,7 +12750,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="277" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>7</v>
       </c>
@@ -12782,7 +12788,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="278" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
         <v>7</v>
       </c>
@@ -12820,7 +12826,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="279" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
         <v>7</v>
       </c>
@@ -12858,7 +12864,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="280" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
         <v>7</v>
       </c>
@@ -12896,7 +12902,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="281" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
         <v>7</v>
       </c>
@@ -12934,7 +12940,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="282" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
         <v>7</v>
       </c>
@@ -12972,7 +12978,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="283" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
         <v>7</v>
       </c>
@@ -13010,7 +13016,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="284" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
         <v>7</v>
       </c>
@@ -13048,7 +13054,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="285" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
         <v>7</v>
       </c>
@@ -13086,7 +13092,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="286" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
         <v>7</v>
       </c>
@@ -13124,7 +13130,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="287" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
         <v>7</v>
       </c>
@@ -13162,7 +13168,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="288" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
         <v>7</v>
       </c>
@@ -13200,7 +13206,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="289" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
         <v>7</v>
       </c>
@@ -13238,7 +13244,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="290" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
         <v>7</v>
       </c>
@@ -13276,7 +13282,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="291" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
         <v>7</v>
       </c>
@@ -13314,7 +13320,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="292" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
         <v>7</v>
       </c>
@@ -13352,7 +13358,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="293" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
         <v>7</v>
       </c>
@@ -13390,7 +13396,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="294" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
         <v>7</v>
       </c>
@@ -13428,7 +13434,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="295" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
         <v>7</v>
       </c>
@@ -13466,7 +13472,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="296" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
         <v>7</v>
       </c>
@@ -13504,7 +13510,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="297" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
         <v>7</v>
       </c>
@@ -13542,7 +13548,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="298" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
         <v>7</v>
       </c>
@@ -13580,7 +13586,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="299" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
         <v>7</v>
       </c>
@@ -13618,7 +13624,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="300" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
         <v>7</v>
       </c>
@@ -13656,7 +13662,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="301" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
         <v>7</v>
       </c>
@@ -13694,7 +13700,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="302" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
         <v>7</v>
       </c>
@@ -13732,7 +13738,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="303" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
         <v>7</v>
       </c>
@@ -13770,7 +13776,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="304" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
         <v>7</v>
       </c>
@@ -13808,7 +13814,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="305" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
         <v>7</v>
       </c>
@@ -13846,7 +13852,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="306" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>7</v>
       </c>
@@ -13884,7 +13890,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="307" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
         <v>7</v>
       </c>
@@ -13922,7 +13928,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="308" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>7</v>
       </c>
@@ -13960,7 +13966,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="309" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
         <v>7</v>
       </c>
@@ -13998,7 +14004,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="310" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
         <v>7</v>
       </c>
@@ -14036,7 +14042,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="311" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
         <v>7</v>
       </c>
@@ -14074,7 +14080,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="312" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
         <v>7</v>
       </c>
@@ -14112,7 +14118,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="313" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
         <v>7</v>
       </c>
@@ -14150,7 +14156,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="314" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
         <v>7</v>
       </c>
@@ -14188,7 +14194,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="315" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
         <v>7</v>
       </c>
@@ -14226,7 +14232,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="316" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
         <v>7</v>
       </c>
@@ -14264,7 +14270,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="317" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
         <v>7</v>
       </c>
@@ -14302,7 +14308,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="318" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
         <v>7</v>
       </c>
@@ -14340,7 +14346,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="319" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
         <v>7</v>
       </c>
@@ -14378,7 +14384,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="320" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
         <v>7</v>
       </c>
@@ -14416,7 +14422,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="321" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
         <v>7</v>
       </c>
@@ -14454,7 +14460,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="322" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
         <v>7</v>
       </c>
@@ -14492,7 +14498,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="323" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
         <v>7</v>
       </c>
@@ -14530,7 +14536,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="324" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
         <v>7</v>
       </c>
@@ -14568,7 +14574,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="325" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
         <v>7</v>
       </c>
@@ -14606,7 +14612,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="326" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
         <v>7</v>
       </c>
@@ -14644,7 +14650,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="327" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
         <v>7</v>
       </c>
@@ -14682,7 +14688,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="328" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
         <v>7</v>
       </c>
@@ -14720,7 +14726,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="329" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
         <v>7</v>
       </c>
@@ -14758,7 +14764,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="330" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
         <v>7</v>
       </c>
@@ -14796,7 +14802,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="331" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
         <v>7</v>
       </c>
@@ -14834,7 +14840,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="332" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
         <v>7</v>
       </c>
@@ -14872,7 +14878,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="333" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
         <v>7</v>
       </c>
@@ -14910,7 +14916,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="334" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
         <v>7</v>
       </c>
@@ -14948,7 +14954,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="335" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
         <v>7</v>
       </c>
@@ -14986,7 +14992,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="336" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
         <v>7</v>
       </c>
@@ -15024,7 +15030,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="337" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
         <v>7</v>
       </c>
@@ -15062,7 +15068,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="338" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
         <v>7</v>
       </c>
@@ -15100,7 +15106,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="339" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
         <v>7</v>
       </c>
@@ -15138,7 +15144,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="340" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
         <v>7</v>
       </c>
@@ -15176,7 +15182,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="341" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
         <v>7</v>
       </c>
@@ -15214,7 +15220,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="342" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
         <v>7</v>
       </c>
@@ -15252,7 +15258,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="343" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
         <v>7</v>
       </c>
@@ -15290,7 +15296,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="344" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
         <v>7</v>
       </c>
@@ -15328,7 +15334,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="345" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
         <v>7</v>
       </c>
@@ -15366,7 +15372,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="346" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
         <v>7</v>
       </c>
@@ -15404,7 +15410,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="347" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
         <v>7</v>
       </c>
@@ -15442,7 +15448,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="348" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
         <v>7</v>
       </c>
@@ -15480,7 +15486,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="349" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
         <v>7</v>
       </c>
@@ -15518,7 +15524,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="350" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
         <v>7</v>
       </c>
@@ -15556,7 +15562,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="351" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
         <v>7</v>
       </c>
@@ -15594,7 +15600,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="352" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
         <v>7</v>
       </c>
@@ -15632,7 +15638,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="353" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
         <v>7</v>
       </c>
@@ -15670,7 +15676,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="354" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
         <v>7</v>
       </c>
@@ -15708,7 +15714,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="355" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
         <v>7</v>
       </c>
@@ -15746,7 +15752,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="356" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
         <v>7</v>
       </c>
@@ -15784,7 +15790,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="357" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
         <v>7</v>
       </c>
@@ -15822,7 +15828,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="358" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
         <v>7</v>
       </c>
@@ -15860,7 +15866,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="359" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
         <v>7</v>
       </c>
@@ -15898,7 +15904,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="360" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
         <v>7</v>
       </c>
@@ -15936,7 +15942,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="361" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
         <v>7</v>
       </c>
@@ -15974,7 +15980,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="362" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
         <v>7</v>
       </c>
@@ -16012,7 +16018,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="363" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
         <v>7</v>
       </c>
@@ -16050,7 +16056,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="364" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
         <v>7</v>
       </c>
@@ -16088,7 +16094,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="365" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
         <v>7</v>
       </c>
@@ -16126,7 +16132,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="366" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
         <v>7</v>
       </c>
@@ -16164,7 +16170,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="367" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
         <v>7</v>
       </c>
@@ -16202,7 +16208,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="368" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
         <v>7</v>
       </c>
@@ -16240,7 +16246,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="369" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
         <v>7</v>
       </c>
@@ -16278,7 +16284,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="370" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
         <v>7</v>
       </c>
@@ -16316,7 +16322,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="371" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
         <v>7</v>
       </c>
@@ -16354,7 +16360,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="372" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
         <v>7</v>
       </c>
@@ -16392,7 +16398,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="373" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
         <v>7</v>
       </c>
@@ -16430,7 +16436,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="374" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
         <v>7</v>
       </c>
@@ -16468,7 +16474,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="375" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
         <v>7</v>
       </c>
@@ -16506,7 +16512,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="376" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
         <v>7</v>
       </c>
@@ -16544,7 +16550,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="377" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
         <v>7</v>
       </c>
@@ -16582,7 +16588,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="378" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
         <v>97</v>
       </c>
@@ -16614,7 +16620,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="379" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
         <v>97</v>
       </c>
@@ -16646,7 +16652,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="380" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
         <v>97</v>
       </c>
@@ -16678,7 +16684,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="381" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
         <v>97</v>
       </c>
@@ -16710,7 +16716,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="382" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
         <v>97</v>
       </c>
@@ -16742,7 +16748,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="383" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
         <v>97</v>
       </c>
@@ -16774,7 +16780,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="384" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
         <v>97</v>
       </c>
@@ -16806,7 +16812,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="385" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
         <v>97</v>
       </c>
@@ -16838,7 +16844,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="386" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
         <v>97</v>
       </c>
@@ -16870,7 +16876,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="387" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
         <v>97</v>
       </c>
@@ -16902,7 +16908,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="388" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
         <v>97</v>
       </c>
@@ -16934,7 +16940,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="389" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
         <v>97</v>
       </c>
@@ -16966,7 +16972,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="390" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
         <v>97</v>
       </c>
@@ -16998,7 +17004,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="391" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
         <v>97</v>
       </c>
@@ -17030,7 +17036,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="392" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
         <v>97</v>
       </c>
@@ -17062,7 +17068,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="393" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
         <v>97</v>
       </c>
@@ -17094,7 +17100,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="394" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
         <v>97</v>
       </c>
@@ -17126,7 +17132,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="395" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
         <v>97</v>
       </c>
@@ -17158,7 +17164,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="396" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
         <v>97</v>
       </c>
@@ -17190,7 +17196,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="397" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
         <v>97</v>
       </c>
@@ -17222,7 +17228,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="398" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
         <v>7</v>
       </c>
@@ -17254,7 +17260,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="399" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
         <v>7</v>
       </c>
@@ -17286,7 +17292,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="400" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
         <v>7</v>
       </c>
@@ -17318,7 +17324,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="401" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
         <v>7</v>
       </c>
@@ -17350,7 +17356,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="402" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
         <v>7</v>
       </c>
@@ -17382,7 +17388,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="403" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
         <v>7</v>
       </c>
@@ -17414,7 +17420,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="404" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
         <v>7</v>
       </c>
@@ -17446,7 +17452,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="405" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
         <v>7</v>
       </c>
@@ -17478,7 +17484,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="406" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
         <v>7</v>
       </c>
@@ -17510,7 +17516,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="407" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
         <v>7</v>
       </c>
@@ -17542,7 +17548,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="408" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="408" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
         <v>7</v>
       </c>
@@ -17574,7 +17580,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="409" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="409" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
         <v>7</v>
       </c>
@@ -17606,7 +17612,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="410" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="410" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
         <v>7</v>
       </c>
@@ -17638,7 +17644,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="411" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="411" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
         <v>7</v>
       </c>
@@ -17670,7 +17676,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="412" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
         <v>7</v>
       </c>
@@ -17702,7 +17708,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="413" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
         <v>7</v>
       </c>
@@ -17734,7 +17740,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="414" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
         <v>7</v>
       </c>
@@ -17766,7 +17772,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="415" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
         <v>7</v>
       </c>
@@ -17798,7 +17804,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="416" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
         <v>7</v>
       </c>
@@ -17830,7 +17836,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="417" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
         <v>7</v>
       </c>
@@ -17862,7 +17868,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="418" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
         <v>7</v>
       </c>
@@ -17894,7 +17900,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="419" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="419" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
         <v>7</v>
       </c>
@@ -17926,7 +17932,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="420" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="420" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
         <v>7</v>
       </c>
@@ -17958,7 +17964,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="421" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="421" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
         <v>7</v>
       </c>
@@ -17990,7 +17996,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="422" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="422" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
         <v>7</v>
       </c>
@@ -18022,7 +18028,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="423" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="423" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
         <v>7</v>
       </c>
@@ -18054,7 +18060,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="424" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="424" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
         <v>7</v>
       </c>
@@ -18086,7 +18092,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="425" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="425" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
         <v>7</v>
       </c>
@@ -18118,7 +18124,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="426" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="426" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
         <v>7</v>
       </c>
@@ -18150,7 +18156,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="427" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="427" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
         <v>7</v>
       </c>
@@ -18188,7 +18194,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="428" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="428" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
         <v>7</v>
       </c>
@@ -18220,7 +18226,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="429" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="429" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
         <v>7</v>
       </c>
@@ -18252,7 +18258,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="430" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="430" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
         <v>7</v>
       </c>
@@ -18284,7 +18290,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="431" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="431" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
         <v>7</v>
       </c>
@@ -18316,7 +18322,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="432" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="432" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
         <v>7</v>
       </c>
@@ -18348,7 +18354,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="433" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="433" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
         <v>7</v>
       </c>
@@ -18380,7 +18386,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="434" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="434" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
         <v>7</v>
       </c>
@@ -18412,7 +18418,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="435" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="435" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A435" t="s">
         <v>7</v>
       </c>
@@ -18444,7 +18450,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="436" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="436" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
         <v>7</v>
       </c>
@@ -18476,7 +18482,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="437" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="437" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
         <v>7</v>
       </c>
@@ -18508,7 +18514,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="438" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="438" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
         <v>7</v>
       </c>
@@ -18540,7 +18546,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="439" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="439" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
         <v>7</v>
       </c>
@@ -18572,7 +18578,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="440" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="440" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A440" t="s">
         <v>7</v>
       </c>
@@ -18604,7 +18610,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="441" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="441" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A441" t="s">
         <v>7</v>
       </c>
@@ -18636,7 +18642,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="442" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="442" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
         <v>7</v>
       </c>
@@ -18668,7 +18674,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="443" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="443" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
         <v>7</v>
       </c>
@@ -18700,7 +18706,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="444" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="444" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
         <v>7</v>
       </c>
@@ -18732,7 +18738,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="445" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="445" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A445" t="s">
         <v>7</v>
       </c>
@@ -18764,7 +18770,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="446" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="446" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
         <v>7</v>
       </c>
@@ -18796,7 +18802,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="447" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="447" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A447" t="s">
         <v>7</v>
       </c>
@@ -18828,7 +18834,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="448" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="448" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
         <v>7</v>
       </c>
@@ -18860,7 +18866,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="449" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="449" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A449" t="s">
         <v>7</v>
       </c>
@@ -18892,7 +18898,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="450" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="450" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
         <v>7</v>
       </c>
@@ -18937,6 +18943,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Criar um novo documento." ma:contentTypeScope="" ma:versionID="9a7078cd21229583650f2264465a1c40">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4e45437c47114f519c494620e3e4bb67" ns2:_="" ns3:_="">
     <xsd:import namespace="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
@@ -19171,27 +19197,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DD773D5-C77E-4BE7-B333-7D7BD35C149E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
+    <ds:schemaRef ds:uri="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{740CB11B-765A-4E9B-962E-5A759873CC55}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0309DC03-8AF9-4F10-8E38-DF287EC74A10}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19208,23 +19233,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{740CB11B-765A-4E9B-962E-5A759873CC55}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DD773D5-C77E-4BE7-B333-7D7BD35C149E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
-    <ds:schemaRef ds:uri="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>